<commit_message>
Refresh: final review fixes, Appendix C robustness check, FYI scripts and models
</commit_message>
<xml_diff>
--- a/Table10_RoBMA_MetaRegression.xlsx
+++ b/Table10_RoBMA_MetaRegression.xlsx
@@ -11,12 +11,13 @@
     <sheet name="Coefficients" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="CommonEstimates" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="PublicationBias" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="AverageStudy" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t xml:space="preserve">Component</t>
   </si>
@@ -33,7 +34,7 @@
     <t xml:space="preserve">Effect</t>
   </si>
   <si>
-    <t xml:space="preserve">204.479452054795</t>
+    <t xml:space="preserve">10.0803324099723</t>
   </si>
   <si>
     <t xml:space="preserve">Heterogeneity</t>
@@ -48,51 +49,12 @@
     <t xml:space="preserve">Moderator</t>
   </si>
   <si>
-    <t xml:space="preserve">SC1_Cognitive</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.0554461018857304</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LaggedDV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.444390948483389</t>
-  </si>
-  <si>
-    <t xml:space="preserve">NumberSCVars</t>
-  </si>
-  <si>
     <t xml:space="preserve">Endog_FE</t>
   </si>
   <si>
-    <t xml:space="preserve">6.32690194162901</t>
-  </si>
-  <si>
     <t xml:space="preserve">Reg_OECDEurope</t>
   </si>
   <si>
-    <t xml:space="preserve">0.175894169524743</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reg_US</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.314405888538381</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reg_Africa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.0609516736512652</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Reg_Asia</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0.117235215253985</t>
-  </si>
-  <si>
     <t xml:space="preserve">Parameter</t>
   </si>
   <si>
@@ -114,6 +76,18 @@
     <t xml:space="preserve">intercept</t>
   </si>
   <si>
+    <t xml:space="preserve">Endog_FE[dif: 0]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Endog_FE[dif: 1]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reg_OECDEurope[dif: 0]</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reg_OECDEurope[dif: 1]</t>
+  </si>
+  <si>
     <t xml:space="preserve">tau</t>
   </si>
   <si>
@@ -142,6 +116,18 @@
   </si>
   <si>
     <t xml:space="preserve">PEESE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quantity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.5%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">97.5%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Average-study bias-corrected mean (Fisher's z)</t>
   </si>
 </sst>
 </file>
@@ -492,7 +478,7 @@
         <v>0.5</v>
       </c>
       <c r="C2" t="n">
-        <v>0.995133333333333</v>
+        <v>0.90975</v>
       </c>
       <c r="D2" t="s">
         <v>5</v>
@@ -559,108 +545,24 @@
         <v>0.5</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0525333333333333</v>
-      </c>
-      <c r="D2" t="s">
-        <v>11</v>
+        <v>0.828066666666667</v>
+      </c>
+      <c r="D2" t="n">
+        <v>4.81620783249321</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B3" t="n">
         <v>0.5</v>
       </c>
       <c r="C3" t="n">
-        <v>0.307666666666667</v>
-      </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>14</v>
-      </c>
-      <c r="B4" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D4" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>15</v>
-      </c>
-      <c r="B5" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C5" t="n">
-        <v>0.863516666666667</v>
-      </c>
-      <c r="D5" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>17</v>
-      </c>
-      <c r="B6" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C6" t="n">
-        <v>0.149583333333333</v>
-      </c>
-      <c r="D6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>19</v>
-      </c>
-      <c r="B7" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.2392</v>
-      </c>
-      <c r="D7" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>21</v>
-      </c>
-      <c r="B8" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.05745</v>
-      </c>
-      <c r="D8" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B9" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0.104933333333333</v>
-      </c>
-      <c r="D9" t="s">
-        <v>24</v>
+        <v>0.123666666666667</v>
+      </c>
+      <c r="D3" t="n">
+        <v>0.141118295930011</v>
       </c>
     </row>
   </sheetData>
@@ -676,79 +578,79 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="B1" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="C1" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="D1" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="E1" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="F1" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>31</v>
+        <v>18</v>
       </c>
       <c r="B2" t="n">
-        <v>0.199969892961571</v>
+        <v>0.0839827282894827</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0307280689099211</v>
+        <v>0.0389174613420451</v>
       </c>
       <c r="D2" t="n">
-        <v>0.140918459717449</v>
+        <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>0.199586715228935</v>
+        <v>0.0880181351756</v>
       </c>
       <c r="F2" t="n">
-        <v>0.262121112615635</v>
+        <v>0.150832355067757</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="B3" t="n">
-        <v>-0.000300763449400815</v>
+        <v>0.0391414182175874</v>
       </c>
       <c r="C3" t="n">
-        <v>0.00690908583723153</v>
+        <v>0.0231804669373955</v>
       </c>
       <c r="D3" t="n">
-        <v>-0.0075344279411987</v>
+        <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>0.0428883802426162</v>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>0.0781435581819071</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="B4" t="n">
-        <v>-0.0325782634619347</v>
+        <v>-0.0391414182175874</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0559549927720286</v>
+        <v>0.0231804669373955</v>
       </c>
       <c r="D4" t="n">
-        <v>-0.174641681980614</v>
+        <v>-0.0781435581819071</v>
       </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>-0.0428883802426162</v>
       </c>
       <c r="F4" t="n">
         <v>0</v>
@@ -756,121 +658,41 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B5" t="n">
-        <v>-0.0334503304168531</v>
+        <v>0.00263044176989667</v>
       </c>
       <c r="C5" t="n">
-        <v>0.00644866456390213</v>
+        <v>0.00987609084451122</v>
       </c>
       <c r="D5" t="n">
-        <v>-0.0460379905936745</v>
+        <v>0</v>
       </c>
       <c r="E5" t="n">
-        <v>-0.0334821233504807</v>
+        <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>-0.0207401132321791</v>
+        <v>0.0363854523421143</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="B6" t="n">
-        <v>-0.0852571939072479</v>
+        <v>-0.00263044176989667</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0443543661405663</v>
+        <v>0.00987609084451122</v>
       </c>
       <c r="D6" t="n">
-        <v>-0.157005015690589</v>
+        <v>-0.0363854523421143</v>
       </c>
       <c r="E6" t="n">
-        <v>-0.0926655366820806</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B7" t="n">
-        <v>-0.00790371015689462</v>
-      </c>
-      <c r="C7" t="n">
-        <v>0.024616904967013</v>
-      </c>
-      <c r="D7" t="n">
-        <v>-0.0923492751769268</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" t="n">
-        <v>-0.0282494660924659</v>
-      </c>
-      <c r="C8" t="n">
-        <v>0.0633951564314822</v>
-      </c>
-      <c r="D8" t="n">
-        <v>-0.21691295068379</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>21</v>
-      </c>
-      <c r="B9" t="n">
-        <v>0.000747223181338244</v>
-      </c>
-      <c r="C9" t="n">
-        <v>0.02379979017003</v>
-      </c>
-      <c r="D9" t="n">
-        <v>-0.00153888673711979</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0.0291333275051826</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" t="n">
-        <v>-0.00735911658624394</v>
-      </c>
-      <c r="C10" t="n">
-        <v>0.0304651480963896</v>
-      </c>
-      <c r="D10" t="n">
-        <v>-0.116872315374656</v>
-      </c>
-      <c r="E10" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -887,62 +709,62 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="B1" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="C1" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="D1" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="E1" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="F1" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="B2" t="n">
-        <v>0.231449311741535</v>
+        <v>0.239226876315776</v>
       </c>
       <c r="C2" t="n">
-        <v>0.0160157000924156</v>
+        <v>0.0163109408588927</v>
       </c>
       <c r="D2" t="n">
-        <v>0.203930751561465</v>
+        <v>0.211110247704357</v>
       </c>
       <c r="E2" t="n">
-        <v>0.23014476491602</v>
+        <v>0.237907175631471</v>
       </c>
       <c r="F2" t="n">
-        <v>0.266721233840305</v>
+        <v>0.274878485198892</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="B3" t="n">
-        <v>0.531336317529004</v>
+        <v>0.5426217025773</v>
       </c>
       <c r="C3" t="n">
-        <v>0.062792668022056</v>
+        <v>0.0606569033537308</v>
       </c>
       <c r="D3" t="n">
-        <v>0.408148312788521</v>
+        <v>0.424320699378044</v>
       </c>
       <c r="E3" t="n">
-        <v>0.531435966772672</v>
+        <v>0.542825037982265</v>
       </c>
       <c r="F3" t="n">
-        <v>0.65374138082957</v>
+        <v>0.659958903740757</v>
       </c>
     </row>
   </sheetData>
@@ -958,27 +780,27 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="B1" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="C1" t="s">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="D1" t="s">
-        <v>28</v>
+        <v>15</v>
       </c>
       <c r="E1" t="s">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="F1" t="s">
-        <v>30</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="B2" t="n">
         <v>1</v>
@@ -998,16 +820,16 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="B3" t="n">
-        <v>0.991922066900788</v>
+        <v>0.991783551416734</v>
       </c>
       <c r="C3" t="n">
-        <v>0.0262908923247387</v>
+        <v>0.0263627585482548</v>
       </c>
       <c r="D3" t="n">
-        <v>0.903886046153622</v>
+        <v>0.902907179127522</v>
       </c>
       <c r="E3" t="n">
         <v>1</v>
@@ -1018,87 +840,87 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="B4" t="n">
-        <v>0.695520058830113</v>
+        <v>0.697384295966272</v>
       </c>
       <c r="C4" t="n">
-        <v>0.0733922379043673</v>
+        <v>0.0747779780416875</v>
       </c>
       <c r="D4" t="n">
-        <v>0.562001320803263</v>
+        <v>0.560986572071128</v>
       </c>
       <c r="E4" t="n">
-        <v>0.691682919112296</v>
+        <v>0.693512906373229</v>
       </c>
       <c r="F4" t="n">
-        <v>0.850541902085971</v>
+        <v>0.853412656078918</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="B5" t="n">
-        <v>0.230506870142248</v>
+        <v>0.231926057080279</v>
       </c>
       <c r="C5" t="n">
-        <v>0.0401526638501573</v>
+        <v>0.0415602368559231</v>
       </c>
       <c r="D5" t="n">
-        <v>0.161237553427129</v>
+        <v>0.159070363439022</v>
       </c>
       <c r="E5" t="n">
-        <v>0.227106634145593</v>
+        <v>0.229016275349548</v>
       </c>
       <c r="F5" t="n">
-        <v>0.318235237916265</v>
+        <v>0.321384417553534</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
       <c r="B6" t="n">
-        <v>0.230506870142248</v>
+        <v>0.231926057080279</v>
       </c>
       <c r="C6" t="n">
-        <v>0.0401526638501573</v>
+        <v>0.0415602368559231</v>
       </c>
       <c r="D6" t="n">
-        <v>0.161237553427129</v>
+        <v>0.159070363439022</v>
       </c>
       <c r="E6" t="n">
-        <v>0.227106634145593</v>
+        <v>0.229016275349548</v>
       </c>
       <c r="F6" t="n">
-        <v>0.318235237916265</v>
+        <v>0.321384417553534</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="B7" t="n">
-        <v>0.230506870142248</v>
+        <v>0.231926057080279</v>
       </c>
       <c r="C7" t="n">
-        <v>0.0401526638501573</v>
+        <v>0.0415602368559231</v>
       </c>
       <c r="D7" t="n">
-        <v>0.161237553427129</v>
+        <v>0.159070363439022</v>
       </c>
       <c r="E7" t="n">
-        <v>0.227106634145593</v>
+        <v>0.229016275349548</v>
       </c>
       <c r="F7" t="n">
-        <v>0.318235237916265</v>
+        <v>0.321384417553534</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="B8" t="n">
         <v>0</v>
@@ -1118,7 +940,7 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="B9" t="n">
         <v>0</v>
@@ -1134,6 +956,45 @@
       </c>
       <c r="F9" t="n">
         <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C1" t="s">
+        <v>34</v>
+      </c>
+      <c r="D1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0.0839827282894827</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>0.150832355067757</v>
       </c>
     </row>
   </sheetData>

</xml_diff>